<commit_message>
Add pitch materials and frontend ad copy updates
- Add pitch deck materials and investor documents
- Add competitive analysis and market research
- Add financial model and founder bio
- Update frontend demo Excel file
- Add frontend ad copy reviewed CSV
- Update gitignore to exclude large media files

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Sonnet 4.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/hyperchexity/demos/07. mRNA Vaccine Permanently Rewrite DNA - X.com Claim/COVID_Vaccine_DNA_Integration_Claims Output.xlsx
+++ b/frontend/hyperchexity/demos/07. mRNA Vaccine Permanently Rewrite DNA - X.com Claim/COVID_Vaccine_DNA_Integration_Claims Output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eliyahuai-my.sharepoint.com/personal/eliyahu_eliyahu_ai/Documents/Desktop/src/perplexityValidator/frontend/hyperchexity/demos/07. mRNA Vaccine Permanently Rewrite DNA - X.com Claim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C089C66-7D27-46C0-BB6E-AE85E9EAA906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{0C089C66-7D27-46C0-BB6E-AE85E9EAA906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81EAD287-192F-47E9-9342-C5DB4468A1CD}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1131" yWindow="0" windowWidth="16869" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Updated Values" sheetId="1" r:id="rId1"/>
@@ -2530,15 +2530,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2844,7 +2852,14 @@
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="13" width="20.69140625" customWidth="1"/>
+    <col min="1" max="2" width="20.69140625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="30.4609375" customWidth="1"/>
+    <col min="4" max="8" width="20.69140625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="61.4609375" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="71.4609375" customWidth="1"/>
+    <col min="11" max="11" width="40" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="20.69140625" customWidth="1"/>
+    <col min="13" max="13" width="80.3046875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.4">
@@ -2888,283 +2903,299 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+    <row r="3" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="H3" t="s">
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+    <row r="4" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H4" t="s">
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
+    <row r="5" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H5" t="s">
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
+    <row r="6" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H6" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+    <row r="7" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="H7" t="s">
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+    <row r="8" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H8" t="s">
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="M8" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+    <row r="9" spans="1:13" ht="104.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="H9" t="s">
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" s="6" t="s">
         <v>94</v>
       </c>
     </row>
@@ -3242,7 +3273,7 @@
       <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3265,7 +3296,7 @@
       <c r="H3" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3288,7 +3319,7 @@
       <c r="H4" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="4" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3311,7 +3342,7 @@
       <c r="H5" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -3334,7 +3365,7 @@
       <c r="H6" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3357,7 +3388,7 @@
       <c r="H7" t="s">
         <v>68</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="3" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3380,7 +3411,7 @@
       <c r="H8" t="s">
         <v>79</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="3" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3403,7 +3434,7 @@
       <c r="H9" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="3" t="s">
         <v>87</v>
       </c>
     </row>

</xml_diff>